<commit_message>
fix(xlsx): generator save ke folder sendiri (sebelumnya ke CWD root) + regenerate status terimplementasi
</commit_message>
<xml_diff>
--- a/docs/api-mapping/api-mapping.xlsx
+++ b/docs/api-mapping/api-mapping.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,14 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
     </font>
     <font>
       <b val="1"/>
@@ -53,7 +61,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +71,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -110,12 +128,20 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -595,7 +621,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -648,9 +674,9 @@
           <t>App.vue (geolocation handler)</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>BEDA-SUMBER</t>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -703,9 +729,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>BELUM</t>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>SEBAGIAN</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -760,7 +786,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -815,7 +841,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -868,7 +894,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -923,7 +949,7 @@
           <t>ForecastTemperatureChart.vue</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -980,7 +1006,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1033,7 +1059,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1088,7 +1114,7 @@
           <t>src/data/cityThemes.ts</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1145,7 +1171,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1200,7 +1226,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1253,9 +1279,9 @@
           <t>WaveRadarMap.vue / MaritimeAdvisorDrawer.vue</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>BELUM</t>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>SEBAGIAN</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1308,7 +1334,7 @@
           <t>TransportWeather.vue</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1363,7 +1389,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1418,7 +1444,7 @@
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1473,7 +1499,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1528,7 +1554,7 @@
           <t>SatelliteMap.vue, WaveRadarMap.vue</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1583,7 +1609,7 @@
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1638,7 +1664,7 @@
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1693,7 +1719,7 @@
           <t>ForecastAirQualityChart.vue</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1748,7 +1774,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1803,7 +1829,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1858,7 +1884,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1913,7 +1939,7 @@
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1968,7 +1994,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2023,7 +2049,7 @@
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -2080,7 +2106,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>BELUM</t>
+          <t>TERIMPLEMENTASI</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2133,7 +2159,7 @@
           <t>EarthquakeActivity.vue, EarthquakeHistory.vue</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2188,7 +2214,7 @@
           <t>App.vue, LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2243,7 +2269,7 @@
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2298,7 +2324,7 @@
           <t>TransportWeather.vue</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2326,7 +2352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2335,7 +2361,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Ringkasan Komparasi API — baseline cuaca.bmkg.go.id (8 Sep 2026) vs project bmkg_cuaca</t>
         </is>
@@ -2359,79 +2385,109 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="n"/>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
+      <c r="A4" s="9" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>TERIMPLEMENTASI</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sudah memanggil API asli &amp; dipakai di UI (fallback mock saat gagal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>SEBAGIAN</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sudah ter-fetch dari API, tapi UI penuh/badge menyusul</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>19</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Endpoint original belum diimplementasikan (data masih mock / fitur belum ada)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="B8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Fitur ada di redesign tapi mengambil data dari sumber berbeda (OSM/OSRM/inderaja/Carto/statik)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sumber yang hanya dipakai redesign (tidak dipakai original)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="C8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Total endpoint terpetakan</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B11" t="n">
         <v>32</v>
       </c>
-      <c r="C9" s="2" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="C11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Endpoint original terimplementasi identik (pakai API yang sama)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B12" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: penanda PROXY vs DIRECT per endpoint (api-mapping.xlsx kolom Akses, catatan-dev-team kolom Akses di Dev, API-MAPPING.md + ENDPOINTS.md)
</commit_message>
<xml_diff>
--- a/docs/api-mapping/api-mapping.xlsx
+++ b/docs/api-mapping/api-mapping.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Mapping'!$A$1:$K$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Mapping'!$A$1:$L$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,6 +35,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00006100"/>
     </font>
     <font>
@@ -51,17 +55,13 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E79"/>
-    </font>
-    <font>
-      <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -75,12 +75,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -128,20 +138,26 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,20 +523,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,25 +573,30 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Akses (dev)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Dipakai di Original (baseline)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Komponen Redesign</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status Redesign</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Sumber Pengganti (Redesign)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Catatan / Response Shape</t>
         </is>
@@ -609,27 +631,32 @@
           <t>Referer+Origin</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Dashboard: cuaca saat ini, prakiraan 10 hari, tab Ringkasan/Per Jam; /perbandingan</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>CurrentWeather.vue, ForecastPanel.vue, ForecastTemperatureChart.vue, ForecastPrecipitationChart.vue, ForecastAirQualityChart.vue</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts (weatherDataMap, hourlyForecastsMap, generateMockWeatherForCity)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Respons: lokasi adm1-adm4 + cuaca per jam &amp; 3-jam hingga +9 hari (t, tcc, tp, weather, wd, ws, hu, vs, image icon). Endpoint paling kritis untuk diimplementasikan.</t>
         </is>
@@ -664,27 +691,32 @@
           <t>Referer+Origin</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Resolve lokasi admin (desa/kec/kotkab/prov) dari koordinat</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>App.vue (geolocation handler)</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Nominatim reverse geocoding (openstreetmap.org)</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Struktur respons original: adm1..adm4 + provinsi/kotkab/kecamatan/desa + timezone. Nominatim butuh mapping manual field-nya.</t>
         </is>
@@ -719,27 +751,32 @@
           <t>Referer+Origin</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Amandemen prakiraan (revisi data)</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>SEBAGIAN</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Fitur belum ada sama sekali di redesign.</t>
         </is>
@@ -774,27 +811,32 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Kartu 'Cuaca Saat Ini' (observasi aktual)</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>CurrentWeather.vue</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts (weatherDataMap)</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Respons: {status, data:{lokasi, cuaca}}.</t>
         </is>
@@ -829,27 +871,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Panel peringatan cuaca wilayah (today/tomorrow)</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>AlertsPanel.vue</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts (warningAlertsMap)</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Respons: {data:{today:{...},tomorrow:{...}}}.</t>
         </is>
@@ -884,27 +931,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Status siklon lokal</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Fitur belum ada.</t>
         </is>
@@ -939,27 +991,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Grafik 'Suhu Mingguan'</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>ForecastTemperatureChart.vue</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Respons: {data:{daily:[{date,temperature}],weekly:[...]}}.</t>
         </is>
@@ -994,27 +1051,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Video Instagram terbaru BMKG</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>NewsSection.vue</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts (newsArticles)</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Respons: array {title, videoUrl, ...}.</t>
         </is>
@@ -1049,27 +1111,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Banner promo di dashboard</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Respons: {data:[{banner}]}. Fitur belum ada.</t>
         </is>
@@ -1104,27 +1171,32 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Tema background per section (public/aviation/maritim)</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>src/data/cityThemes.ts</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Tema statis lokal</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Bebas auth; nilai setting.background bisa dipakai untuk dinamisasi tema.</t>
         </is>
@@ -1159,27 +1231,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Info matahari &amp; bulan (30+ field: sunrise, golden_hour, moon_phase, dll)</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>CurrentWeather.vue (sunrise/sunset untuk day/night)</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Data statis/mock</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Bisa replace dengan perhitungan lokal (mis. SunCalc) ATAU langsung endpoint ini.</t>
         </is>
@@ -1214,27 +1291,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Sirkulasi siklon TCWC Jakarta</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Respons: {status, data:{cyclone_info:[...]}}.</t>
         </is>
@@ -1269,27 +1351,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Wilayah laut terdekat (drawer maritim)</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>WaveRadarMap.vue / MaritimeAdvisorDrawer.vue</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>SEBAGIAN</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Respons: {data:{code:'F.09', name:'Teluk Jakarta', wilpel, geometry:Polygon}}.</t>
         </is>
@@ -1324,27 +1411,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Rute pelayaran maritim</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>TransportWeather.vue</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>OSRM (router.project-osrm.org)</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>404 via Node, 200 via browser (butuh context CF).</t>
         </is>
@@ -1379,27 +1471,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>GeoJSON titik area laut</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1434,27 +1531,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Katalog run model (radar/windmap)</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>inderaja.bmkg.go.id/IMAGE/HIMA/*.png (statis)</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Original pakai ini + spartan untuk layer dinamis.</t>
         </is>
@@ -1489,27 +1591,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Impact-Based Forecast per tanggal (/ibf + layer Peringatan /map)</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Fitur IBF belum ada di redesign.</t>
         </is>
@@ -1544,27 +1651,32 @@
           <t>campuran</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Metadata layer peta (sources, layers, overlays)</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>SatelliteMap.vue, WaveRadarMap.vue</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>CartoCDN basemap (basemaps.cartocdn.com)</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>warning/maritim terbuka; general/aviation/tourism perlu X-API-KEY.</t>
         </is>
@@ -1599,27 +1711,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>POI wisata (layer Turis /map)</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Overpass API (OSM)</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1654,27 +1771,32 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>POI layer umum /map</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Overpass API (OSM)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>502 flaky saat probe; 200 via browser.</t>
         </is>
@@ -1709,27 +1831,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Tile peta polusi (layer Peringatan /map)</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>ForecastAirQualityChart.vue</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>AQ chart redesign pakai data mock.</t>
         </is>
@@ -1764,27 +1891,32 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Tipe subscription (/premium)</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Halaman premium belum ada di redesign.</t>
         </is>
@@ -1819,27 +1951,32 @@
           <t>Akun dev</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Console developer (/devtools, /Login, /register)</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Tidak relevan untuk redesign publik (opsional).</t>
         </is>
@@ -1874,27 +2011,32 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Katalog model (gfs_indo, spartan, pcm_pm25, QPE, FDRS, dll)</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Respons kaya (14+ katalog model) — potensi untuk layer radar/iklim.</t>
         </is>
@@ -1929,27 +2071,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Data satelit CGMS</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>inderaja.bmkg.go.id/IMAGE/HIMA/*.png</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>404 tanpa param; butuh reverse-engineering param dari browser.</t>
         </is>
@@ -1984,27 +2131,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Tile angin ECMWF</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>Wind layer belum ada di redesign.</t>
         </is>
@@ -2039,27 +2191,32 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Boundary administratif peta</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>CartoCDN basemap</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2094,27 +2251,32 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Konten /berita, /berita/infografis, /berita/video (SSR)</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>NewsSection.vue</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>src/data/mockData.ts (newsArticles)</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>WP REST API standar — mudah diintegrasikan.</t>
         </is>
@@ -2149,27 +2311,32 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>TIDAK ADA di original (cuaca.bmkg.go.id tidak menampilkan gempa)</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>EarthquakeActivity.vue, EarthquakeHistory.vue</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
+      <c r="J30" s="9" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Legacy BMKG endpoint; dipakai redesign sebagai fitur tambahan.</t>
         </is>
@@ -2204,27 +2371,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>TIDAK ADA di original</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>App.vue, LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="J31" s="9" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>Pengganti adm/coord + pencarian lokasi.</t>
         </is>
@@ -2259,27 +2431,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>TIDAK ADA di original</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="J32" s="9" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>POI aktivitas darat.</t>
         </is>
@@ -2314,34 +2491,39 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>TIDAK ADA di original</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>TransportWeather.vue</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="J33" s="9" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
           <t>Routing transportasi darat.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K33"/>
+  <autoFilter ref="A1:L33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2361,7 +2543,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Ringkasan Komparasi API — baseline cuaca.bmkg.go.id (8 Sep 2026) vs project bmkg_cuaca</t>
         </is>
@@ -2385,12 +2567,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="9" t="n"/>
-      <c r="C4" s="9" t="n"/>
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -2405,7 +2587,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>SEBAGIAN</t>
         </is>
@@ -2420,7 +2602,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2435,7 +2617,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -2450,7 +2632,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2479,7 +2661,7 @@
       <c r="C11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Endpoint original terimplementasi identik (pakai API yang sama)</t>
         </is>

</xml_diff>